<commit_message>
Regenerate artifacts for the NucleicAcid entity
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/excel/lambda_ber_schema.xlsx
+++ b/assets/excel/lambda_ber_schema.xlsx
@@ -33,62 +33,64 @@
     <sheet name="Sample" sheetId="24" state="visible" r:id="rId24"/>
     <sheet name="Protein" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="ProteinConstruct" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="SamplePreparation" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Instrument" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="CryoEMInstrument" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="XRayInstrument" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="SANSDetector" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="SANSSource" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="SANSConfiguration" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="SANSInstrument" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="SAXSInstrument" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet name="BeamlineInstrument" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="ExperimentRun" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="WorkflowRun" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet name="DataFile" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet name="Image" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet name="Image2D" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet name="Image3D" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="Movie" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="Micrograph" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet name="FTIRImage" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet name="FluorescenceImage" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet name="OpticalImage" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet name="XRFImage" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet name="ImageFeature" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet name="OntologyTerm" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet name="MolecularComposition" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet name="BufferComposition" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet name="StorageConditions" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet name="CryoEMPreparation" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet name="CrystallizationConditions" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet name="XRayPreparation" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet name="SAXSPreparation" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet name="ExperimentalConditions" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet name="DataCollectionStrategy" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet name="BeamCenterPixels" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet name="QualityMetrics" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet name="ComputeResources" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet name="CryoEMQualityMetrics" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet name="MotionCorrectionParameters" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet name="CTFEstimationParameters" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet name="ParticlePickingParameters" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet name="RefinementParameters" sheetId="67" state="visible" r:id="rId67"/>
-    <sheet name="FSCCurve" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet name="StudySampleAssociation" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet name="StudyExperimentAssociation" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet name="StudyWorkflowAssociation" sheetId="71" state="visible" r:id="rId71"/>
-    <sheet name="ExperimentSampleAssociation" sheetId="72" state="visible" r:id="rId72"/>
-    <sheet name="SampleProteinAssociation" sheetId="73" state="visible" r:id="rId73"/>
-    <sheet name="ExperimentInstrumentAssociation" sheetId="74" state="visible" r:id="rId74"/>
-    <sheet name="WorkflowExperimentAssociation" sheetId="75" state="visible" r:id="rId75"/>
-    <sheet name="WorkflowInputAssociation" sheetId="76" state="visible" r:id="rId76"/>
-    <sheet name="WorkflowOutputAssociation" sheetId="77" state="visible" r:id="rId77"/>
-    <sheet name="StudyPersonAssociation" sheetId="78" state="visible" r:id="rId78"/>
-    <sheet name="ExperimentPersonAssociation" sheetId="79" state="visible" r:id="rId79"/>
-    <sheet name="WorkflowPersonAssociation" sheetId="80" state="visible" r:id="rId80"/>
-    <sheet name="StudyOrganizationAssociation" sheetId="81" state="visible" r:id="rId81"/>
-    <sheet name="PersonOrganizationAssociation" sheetId="82" state="visible" r:id="rId82"/>
+    <sheet name="NucleicAcid" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="SamplePreparation" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Instrument" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="CryoEMInstrument" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="XRayInstrument" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="SANSDetector" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="SANSSource" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="SANSConfiguration" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="SANSInstrument" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="SAXSInstrument" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="BeamlineInstrument" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="ExperimentRun" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="WorkflowRun" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="DataFile" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="Image" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="Image2D" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="Image3D" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="Movie" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="Micrograph" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="FTIRImage" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="FluorescenceImage" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="OpticalImage" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="XRFImage" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="ImageFeature" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="OntologyTerm" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="MolecularComposition" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="BufferComposition" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="StorageConditions" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="CryoEMPreparation" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="CrystallizationConditions" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet name="XRayPreparation" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="SAXSPreparation" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet name="ExperimentalConditions" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet name="DataCollectionStrategy" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet name="BeamCenterPixels" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet name="QualityMetrics" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet name="ComputeResources" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet name="CryoEMQualityMetrics" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet name="MotionCorrectionParameters" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="CTFEstimationParameters" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet name="ParticlePickingParameters" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet name="RefinementParameters" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet name="FSCCurve" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet name="StudySampleAssociation" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet name="StudyExperimentAssociation" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="StudyWorkflowAssociation" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet name="ExperimentSampleAssociation" sheetId="73" state="visible" r:id="rId73"/>
+    <sheet name="SampleProteinAssociation" sheetId="74" state="visible" r:id="rId74"/>
+    <sheet name="SampleNucleicAcidAssociation" sheetId="75" state="visible" r:id="rId75"/>
+    <sheet name="ExperimentInstrumentAssociation" sheetId="76" state="visible" r:id="rId76"/>
+    <sheet name="WorkflowExperimentAssociation" sheetId="77" state="visible" r:id="rId77"/>
+    <sheet name="WorkflowInputAssociation" sheetId="78" state="visible" r:id="rId78"/>
+    <sheet name="WorkflowOutputAssociation" sheetId="79" state="visible" r:id="rId79"/>
+    <sheet name="StudyPersonAssociation" sheetId="80" state="visible" r:id="rId80"/>
+    <sheet name="ExperimentPersonAssociation" sheetId="81" state="visible" r:id="rId81"/>
+    <sheet name="WorkflowPersonAssociation" sheetId="82" state="visible" r:id="rId82"/>
+    <sheet name="StudyOrganizationAssociation" sheetId="83" state="visible" r:id="rId83"/>
+    <sheet name="PersonOrganizationAssociation" sheetId="84" state="visible" r:id="rId84"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1137,7 +1139,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"uniprot,pdb,pfam,cath,scop,interpro,chembl,chebi,pubchem,drugbank,omim,clinvar,cosmic,gnomad,intact,string,biogrid,reactome,kegg,go"</formula1>
+      <formula1>"uniprot,pdb,pfam,cath,scop,interpro,chembl,chebi,pubchem,drugbank,omim,clinvar,cosmic,gnomad,intact,string,biogrid,reactome,kegg,go,rnacentral,rfam,refseq,insdc,mirbase,gtrnadb,ndb,modomics"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1454,7 +1456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD1"/>
+  <dimension ref="A1:AF1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1495,115 +1497,125 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>nucleic_acids</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>samples</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>sample_preparations</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>experiment_runs</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>workflow_runs</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>data_files</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>images</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>study_sample_associations</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>study_experiment_associations</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>study_workflow_associations</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>experiment_sample_associations</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>experiment_instrument_associations</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>sample_protein_associations</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>sample_nucleic_acid_associations</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
         <is>
           <t>workflow_experiment_associations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>workflow_input_associations</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>workflow_output_associations</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>study_person_associations</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>experiment_person_associations</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>workflow_person_associations</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>study_organization_associations</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>person_organization_associations</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -2307,6 +2319,117 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:R1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>nucleic_acid_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>nucleic_acid_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>rnacentral_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>sequence_accession</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>rfam_families</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>gene_name</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>organism</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>organism_name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>nucleotide_sequence</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>sequence_length</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>molecular_weight_theoretical</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>function_description</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>go_terms</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>pdb_entries</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>cross_references</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"dna,rna,dna_rna_hybrid,peptide_nucleic_acid,other"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AS1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -2553,7 +2676,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2650,7 +2773,58 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>maximum_numeric_value</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>minimum_numeric_value</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>numeric_value</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>unit_cv_id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>attribute</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>raw_value</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2886,58 +3060,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>maximum_numeric_value</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>minimum_numeric_value</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>numeric_value</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>unit_cv_id</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>attribute</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>raw_value</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3100,7 +3223,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3171,7 +3294,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3227,7 +3350,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3308,7 +3431,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3443,7 +3566,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3570,7 +3693,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3742,7 +3865,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4150,7 +4273,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4511,7 +4634,43 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>value_cv_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>attribute</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>raw_value</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4600,98 +4759,698 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>value_cv_id</t>
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>acquisition_date</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>attribute</t>
+          <t>pixel_size</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>raw_value</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+          <t>dimensions_x</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>dimensions_y</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>exposure_time</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>defocus</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>astigmatism</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
         <is>
           <t>file_name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>acquisition_date</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>pixel_size</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>dimensions_x</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>dimensions_y</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>exposure_time</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>dimensions_z</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>voxel_size</t>
+        </is>
+      </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>reconstruction_method</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>acquisition_date</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>pixel_size</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>dimensions_x</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>dimensions_y</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>exposure_time</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AA1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>frames</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>super_resolution</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>pixel_size_unbinned</t>
+        </is>
+      </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>stage_position_x</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>stage_position_y</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>stage_position_z</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>nominal_defocus</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>dose_per_frame</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>beam_shift_x</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>beam_shift_y</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ice_thickness_estimate</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>grid_square_id</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>hole_id</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>acquisition_group</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>defocus</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>astigmatism</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>acquisition_date</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>pixel_size</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
           <t>dimensions_x</t>
         </is>
       </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>dimensions_y</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>exposure_time</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>origin_movie_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>defocus_u</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>defocus_v</t>
+        </is>
+      </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>astigmatism_angle</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>resolution_fit_limit</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>ctf_quality_score</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>defocus</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>astigmatism</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>acquisition_date</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>pixel_size</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>dimensions_x</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>dimensions_y</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>exposure_time</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>wavenumber_min</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>wavenumber_max</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>spectral_resolution</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>number_of_scans</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>apodization_function</t>
+        </is>
+      </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>molecular_signatures</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>background_correction</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>acquisition_date</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>pixel_size</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>dimensions_x</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>dimensions_y</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>exposure_time</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>dose</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>excitation_wavelength</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>emission_wavelength</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>excitation_filter</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>emission_filter</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>fluorophore</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>channel_name</t>
+        </is>
+      </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>laser_power</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>pinhole_size</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>quantum_yield</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>defocus</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>astigmatism</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>file_name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>acquisition_date</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>pixel_size</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>dimensions_x</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>dimensions_y</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>exposure_time</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
           <t>dose</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -4702,643 +5461,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>defocus</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>astigmatism</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>file_name</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>acquisition_date</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>pixel_size</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>dimensions_x</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>dimensions_y</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>exposure_time</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>dose</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>dimensions_z</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>voxel_size</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>reconstruction_method</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>file_name</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>acquisition_date</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>pixel_size</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>dimensions_x</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>dimensions_y</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>exposure_time</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>dose</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AA1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>frames</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>super_resolution</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>pixel_size_unbinned</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>timestamp</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>stage_position_x</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>stage_position_y</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>stage_position_z</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>nominal_defocus</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>dose_per_frame</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>beam_shift_x</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>beam_shift_y</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>ice_thickness_estimate</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>grid_square_id</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>hole_id</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>acquisition_group</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>defocus</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>astigmatism</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>file_name</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>acquisition_date</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>pixel_size</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>dimensions_x</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>dimensions_y</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>exposure_time</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>dose</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:R1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>dose</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>origin_movie_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>defocus_u</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>defocus_v</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>astigmatism_angle</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>resolution_fit_limit</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>ctf_quality_score</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>defocus</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>astigmatism</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>file_name</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>acquisition_date</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>pixel_size</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>dimensions_x</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>dimensions_y</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>exposure_time</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Q1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>wavenumber_min</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>wavenumber_max</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>spectral_resolution</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>number_of_scans</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>apodization_function</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>molecular_signatures</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>background_correction</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>file_name</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>acquisition_date</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>pixel_size</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>dimensions_x</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>dimensions_y</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>exposure_time</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>dose</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:U1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>excitation_wavelength</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>emission_wavelength</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>excitation_filter</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>emission_filter</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>fluorophore</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>channel_name</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>laser_power</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>pinhole_size</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>quantum_yield</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>defocus</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>astigmatism</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>file_name</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>acquisition_date</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>pixel_size</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>dimensions_x</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>dimensions_y</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>exposure_time</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>dose</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5449,7 +5572,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5578,7 +5701,38 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>attribute</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>raw_value</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5604,79 +5758,84 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>attribute</t>
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>terms</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>label</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>raw_value</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>terms</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>label</t>
+          <t>definition</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ontology</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sequences</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>modifications</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>definition</t>
+          <t>ligands</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>ontology</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
           <t>description</t>
         </is>
       </c>
@@ -5686,7 +5845,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5698,17 +5857,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>sequences</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>modifications</t>
+          <t>ph</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>components</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>ligands</t>
+          <t>additives</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -5722,7 +5881,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5734,17 +5893,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ph</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>components</t>
+          <t>temperature</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>duration</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>additives</t>
+          <t>atmosphere</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -5758,43 +5917,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>temperature</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>duration</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>atmosphere</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5936,7 +6059,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6027,7 +6150,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6178,7 +6301,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6224,7 +6347,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6275,7 +6398,93 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>protein_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>pdb_entry</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>chain_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>residue_range</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>confidence_score</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>evidence_type</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>evidence_code</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>source_database</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>annotation_method</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>publication_ids</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"experimental,predicted,inferred,literature,author_statement,curator_inference"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6424,114 +6633,255 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>protein_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>pdb_entry</t>
+<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>xbeam</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ybeam</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>chain_id</t>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AH1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>resolution</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>resolution_high_shell_a</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>resolution_low_a</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>residue_range</t>
+          <t>completeness</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>confidence_score</t>
+          <t>completeness_high_res_shell_percent</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>evidence_type</t>
+          <t>signal_to_noise</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>evidence_code</t>
+          <t>mean_i_over_sigma_i</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>source_database</t>
+          <t>space_group</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>annotation_method</t>
+          <t>unit_cell_a</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>publication_ids</t>
+          <t>unit_cell_b</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>unit_cell_c</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>title</t>
+          <t>unit_cell_alpha</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>unit_cell_beta</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>unit_cell_gamma</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>multiplicity</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>cc_half</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>r_merge</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>r_pim</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>wilson_b_factor_a2</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>anomalous_used</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>anom_corr</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>anom_sig_ano</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>r_work</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>r_free</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>ramachandran_favored_percent</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>ramachandran_outliers_percent</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>clashscore</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>molprobity_score</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>average_b_factor_a2</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>i_zero</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>rg</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>grid_quality</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>r_factor</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"experimental,predicted,inferred,literature,author_statement,curator_inference"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet60.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>xbeam</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>ybeam</t>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>cpu_hours</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>gpu_hours</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>memory_gb</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>storage_gb</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
@@ -6541,234 +6891,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AH1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>resolution</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>resolution_high_shell_a</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>resolution_low_a</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>completeness</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>completeness_high_res_shell_percent</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>signal_to_noise</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>mean_i_over_sigma_i</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>space_group</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>unit_cell_a</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>unit_cell_b</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>unit_cell_c</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>unit_cell_alpha</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>unit_cell_beta</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>unit_cell_gamma</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>multiplicity</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>cc_half</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>r_merge</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>r_pim</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>wilson_b_factor_a2</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>anomalous_used</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>anom_corr</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>anom_sig_ano</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>r_work</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>r_free</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>ramachandran_favored_percent</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>ramachandran_outliers_percent</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>clashscore</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>molprobity_score</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>average_b_factor_a2</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>i_zero</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>rg</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>grid_quality</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
-        <is>
-          <t>r_factor</t>
-        </is>
-      </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>cpu_hours</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>gpu_hours</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>memory_gb</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>storage_gb</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6815,7 +6938,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6876,7 +6999,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6927,7 +7050,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6988,7 +7111,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7054,7 +7177,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7085,7 +7208,133 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>site_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>site_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>residues</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ligand_interactions</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>conservation_score</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>functional_importance</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>go_terms</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>ec_number</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>protein_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>pdb_entry</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>chain_id</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>residue_range</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>confidence_score</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>evidence_type</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>evidence_code</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>source_database</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>annotation_method</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>publication_ids</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="N2:N1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"experimental,predicted,inferred,literature,author_statement,curator_inference"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7126,133 +7375,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:U1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>site_type</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>site_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>residues</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>ligand_interactions</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>conservation_score</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>functional_importance</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>go_terms</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>ec_number</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>protein_id</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>pdb_entry</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>chain_id</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>residue_range</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>confidence_score</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>evidence_type</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>evidence_code</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>source_database</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>annotation_method</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>publication_ids</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="N2:N1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"experimental,predicted,inferred,literature,author_statement,curator_inference"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7278,7 +7401,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7304,7 +7427,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7345,7 +7468,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7416,7 +7539,89 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sample_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>nucleic_acid_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>copy_number</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>residue_range</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>sequence_coverage</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>chain_ids</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>structural_form</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>source_method</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>modifications</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>observed_molecular_weight</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"target,subunit,binding_partner,template,primer,guide,scaffold,contaminant,standard"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"single_stranded,double_stranded,hairpin,triplex,quadruplex,junction,circular,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"chemical_synthesis,in_vitro_transcription,pcr_amplification,plasmid_preparation,isolated_from_organism,other"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7452,7 +7657,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7478,7 +7683,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7514,7 +7719,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7550,7 +7755,147 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>feature_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>secondary_structure</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>solvent_accessibility</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>backbone_flexibility</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>disorder_probability</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>conformational_state</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>structural_motif</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>domain_assignment</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>domain_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>protein_id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>pdb_entry</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>chain_id</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>residue_range</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>confidence_score</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>evidence_type</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>evidence_code</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>source_database</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>annotation_method</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>publication_ids</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="4">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"alpha_helix,beta_sheet,beta_strand,turn,coil,disordered_region,transmembrane_helix,signal_peptide,transit_peptide,domain,repeat,zinc_finger,zinc_binding,coiled_coil,motif,cavity,channel,pore,hinge,linker"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"helix,sheet,turn,coil,helix_310,helix_pi,bend,bridge"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"open,closed,intermediate,active,inactive,apo,holo,substrate_bound,product_bound,inhibitor_bound,partially_open,partially_closed,disordered"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"experimental,predicted,inferred,literature,author_statement,curator_inference"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet80.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7596,7 +7941,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet81.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7632,147 +7977,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:V1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>feature_type</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>secondary_structure</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>solvent_accessibility</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>backbone_flexibility</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>disorder_probability</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>conformational_state</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>structural_motif</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>domain_assignment</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>domain_id</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>protein_id</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>pdb_entry</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>chain_id</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>residue_range</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>confidence_score</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>evidence_type</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>evidence_code</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>source_database</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>annotation_method</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>publication_ids</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="4">
-    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"alpha_helix,beta_sheet,beta_strand,turn,coil,disordered_region,transmembrane_helix,signal_peptide,transit_peptide,domain,repeat,zinc_finger,zinc_binding,coiled_coil,motif,cavity,channel,pore,hinge,linker"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"helix,sheet,turn,coil,helix_310,helix_pi,bend,bridge"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"open,closed,intermediate,active,inactive,apo,holo,substrate_bound,product_bound,inhibitor_bound,partially_open,partially_closed,disordered"</formula1>
-    </dataValidation>
-    <dataValidation sqref="O2:O1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"experimental,predicted,inferred,literature,author_statement,curator_inference"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet80.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet82.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7808,7 +8013,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet81.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet83.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7849,7 +8054,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet82.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet84.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Regenerate artifacts for the sample component tables
Also picks up the Cas9 example, whose source had changed after its
generated copies were last written, and the version line
uv-dynamic-versioning manages in the schema header.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/excel/lambda_ber_schema.xlsx
+++ b/assets/excel/lambda_ber_schema.xlsx
@@ -34,63 +34,66 @@
     <sheet name="Protein" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="ProteinConstruct" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="NucleicAcid" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="SamplePreparation" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Instrument" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="CryoEMInstrument" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="XRayInstrument" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="SANSDetector" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="SANSSource" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="SANSConfiguration" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="SANSInstrument" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet name="SAXSInstrument" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="BeamlineInstrument" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="ExperimentRun" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet name="WorkflowRun" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet name="DataFile" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet name="Image" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet name="Image2D" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="Image3D" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="Movie" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet name="Micrograph" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet name="FTIRImage" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet name="FluorescenceImage" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet name="OpticalImage" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet name="XRFImage" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet name="ImageFeature" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet name="OntologyTerm" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet name="MolecularComposition" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet name="BufferComposition" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet name="StorageConditions" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet name="CryoEMPreparation" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet name="CrystallizationConditions" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet name="XRayPreparation" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet name="SAXSPreparation" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet name="ExperimentalConditions" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet name="DataCollectionStrategy" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet name="BeamCenterPixels" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet name="QualityMetrics" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet name="ComputeResources" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet name="CryoEMQualityMetrics" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet name="MotionCorrectionParameters" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet name="CTFEstimationParameters" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet name="ParticlePickingParameters" sheetId="67" state="visible" r:id="rId67"/>
-    <sheet name="RefinementParameters" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet name="FSCCurve" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet name="StudySampleAssociation" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet name="StudyExperimentAssociation" sheetId="71" state="visible" r:id="rId71"/>
-    <sheet name="StudyWorkflowAssociation" sheetId="72" state="visible" r:id="rId72"/>
-    <sheet name="ExperimentSampleAssociation" sheetId="73" state="visible" r:id="rId73"/>
-    <sheet name="SampleProteinAssociation" sheetId="74" state="visible" r:id="rId74"/>
-    <sheet name="SampleNucleicAcidAssociation" sheetId="75" state="visible" r:id="rId75"/>
-    <sheet name="ExperimentInstrumentAssociation" sheetId="76" state="visible" r:id="rId76"/>
-    <sheet name="WorkflowExperimentAssociation" sheetId="77" state="visible" r:id="rId77"/>
-    <sheet name="WorkflowInputAssociation" sheetId="78" state="visible" r:id="rId78"/>
-    <sheet name="WorkflowOutputAssociation" sheetId="79" state="visible" r:id="rId79"/>
-    <sheet name="StudyPersonAssociation" sheetId="80" state="visible" r:id="rId80"/>
-    <sheet name="ExperimentPersonAssociation" sheetId="81" state="visible" r:id="rId81"/>
-    <sheet name="WorkflowPersonAssociation" sheetId="82" state="visible" r:id="rId82"/>
-    <sheet name="StudyOrganizationAssociation" sheetId="83" state="visible" r:id="rId83"/>
-    <sheet name="PersonOrganizationAssociation" sheetId="84" state="visible" r:id="rId84"/>
+    <sheet name="SmallMolecule" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="SampleComponent" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="SamplePreparation" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Instrument" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="CryoEMInstrument" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="XRayInstrument" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="SANSDetector" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="SANSSource" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="SANSConfiguration" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="SANSInstrument" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="SAXSInstrument" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="BeamlineInstrument" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="ExperimentRun" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="WorkflowRun" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="DataFile" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="Image" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="Image2D" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="Image3D" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="Movie" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="Micrograph" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="FTIRImage" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="FluorescenceImage" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="OpticalImage" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="XRFImage" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="ImageFeature" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="OntologyTerm" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="MolecularComposition" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="BufferComposition" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="StorageConditions" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet name="CryoEMPreparation" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="CrystallizationConditions" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet name="XRayPreparation" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet name="SAXSPreparation" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet name="ExperimentalConditions" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet name="DataCollectionStrategy" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet name="BeamCenterPixels" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet name="QualityMetrics" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet name="ComputeResources" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="CryoEMQualityMetrics" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet name="MotionCorrectionParameters" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet name="CTFEstimationParameters" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet name="ParticlePickingParameters" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet name="RefinementParameters" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet name="FSCCurve" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="StudySampleAssociation" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet name="StudyExperimentAssociation" sheetId="73" state="visible" r:id="rId73"/>
+    <sheet name="StudyWorkflowAssociation" sheetId="74" state="visible" r:id="rId74"/>
+    <sheet name="ExperimentSampleAssociation" sheetId="75" state="visible" r:id="rId75"/>
+    <sheet name="SampleProteinAssociation" sheetId="76" state="visible" r:id="rId76"/>
+    <sheet name="SampleNucleicAcidAssociation" sheetId="77" state="visible" r:id="rId77"/>
+    <sheet name="SampleComponentInteraction" sheetId="78" state="visible" r:id="rId78"/>
+    <sheet name="ExperimentInstrumentAssociation" sheetId="79" state="visible" r:id="rId79"/>
+    <sheet name="WorkflowExperimentAssociation" sheetId="80" state="visible" r:id="rId80"/>
+    <sheet name="WorkflowInputAssociation" sheetId="81" state="visible" r:id="rId81"/>
+    <sheet name="WorkflowOutputAssociation" sheetId="82" state="visible" r:id="rId82"/>
+    <sheet name="StudyPersonAssociation" sheetId="83" state="visible" r:id="rId83"/>
+    <sheet name="ExperimentPersonAssociation" sheetId="84" state="visible" r:id="rId84"/>
+    <sheet name="WorkflowPersonAssociation" sheetId="85" state="visible" r:id="rId85"/>
+    <sheet name="StudyOrganizationAssociation" sheetId="86" state="visible" r:id="rId86"/>
+    <sheet name="PersonOrganizationAssociation" sheetId="87" state="visible" r:id="rId87"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1456,7 +1459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AI1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1502,120 +1505,135 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>small_molecules</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>samples</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>sample_components</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
         <is>
           <t>sample_preparations</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>experiment_runs</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>workflow_runs</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>data_files</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>images</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>study_sample_associations</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>study_experiment_associations</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>study_workflow_associations</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>experiment_sample_associations</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>experiment_instrument_associations</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>sample_protein_associations</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>sample_nucleic_acid_associations</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>sample_component_interactions</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
         <is>
           <t>workflow_experiment_associations</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>workflow_input_associations</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>workflow_output_associations</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>study_person_associations</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>experiment_person_associations</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>workflow_person_associations</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>study_organization_associations</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>person_organization_associations</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -2024,7 +2042,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"protein,nucleic_acid,complex,membrane_protein,virus,organelle"</formula1>
+      <formula1>"protein,nucleic_acid,complex,membrane_protein,virus,organelle,cell,tissue"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2430,6 +2448,227 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>small_molecule_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>chebi_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>pdb_ligand_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>chemical_class</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>molecular_formula</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>smiles</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>inchi</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>inchikey</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>molecular_weight_theoretical</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>cross_references</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ion,lipid,detergent,carbohydrate,nucleotide,amino_acid,organic,polymer,other"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sample_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>component_type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>protein_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>nucleic_acid_id</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>small_molecule_id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ontology_term</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>copy_number</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>concentration</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"protein,nucleic_acid,small_molecule,virus_particle,organelle,cell,tissue,membrane_mimetic,nanoparticle,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"target,subunit,binding_partner,ligand,substrate,product,inhibitor,activator,cofactor,fusion_partner,chaperone,template,primer,guide,scaffold,carrier,additive,contaminant,standard"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>maximum_numeric_value</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>minimum_numeric_value</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>numeric_value</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>unit_cv_id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>attribute</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>raw_value</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AS1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -2676,7 +2915,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2773,58 +3012,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>maximum_numeric_value</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>minimum_numeric_value</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>numeric_value</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>unit_cv_id</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>attribute</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>raw_value</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3060,7 +3248,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3223,7 +3411,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3294,7 +3482,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3350,7 +3538,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3431,7 +3619,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3566,7 +3754,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3693,7 +3881,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3865,7 +4053,43 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>value_cv_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>attribute</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>raw_value</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4273,7 +4497,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4634,43 +4858,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>value_cv_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>attribute</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>raw_value</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4759,7 +4947,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4825,7 +5013,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4901,7 +5089,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4982,7 +5170,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5133,7 +5321,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5239,7 +5427,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5340,7 +5528,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5461,7 +5649,38 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>attribute</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>raw_value</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5572,7 +5791,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5701,53 +5920,73 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>attribute</t>
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>terms</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>terms</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>label</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>raw_value</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>terms</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
+          <t>definition</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ontology</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -5758,48 +5997,33 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>terms</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>label</t>
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sequences</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>modifications</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>definition</t>
+          <t>ligands</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>ontology</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
           <t>description</t>
         </is>
       </c>
@@ -5809,7 +6033,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5821,17 +6045,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>sequences</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>modifications</t>
+          <t>ph</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>components</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>ligands</t>
+          <t>additives</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -5845,7 +6069,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5857,17 +6081,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ph</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>components</t>
+          <t>temperature</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>duration</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>additives</t>
+          <t>atmosphere</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -5881,43 +6105,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>temperature</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>duration</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>atmosphere</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6059,7 +6247,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6150,7 +6338,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6301,103 +6489,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet58.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>concentration_series</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>buffer_matching_protocol</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>sample_cell_type</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>cell_path_length</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>temperature_control</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet59.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>temperature</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>humidity</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>pressure</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>atmosphere</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>beam_energy</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>exposure_time</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -6490,6 +6581,103 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>concentration_series</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>buffer_matching_protocol</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>sample_cell_type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>cell_path_length</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>temperature_control</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>temperature</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>humidity</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>pressure</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>atmosphere</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>beam_energy</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>exposure_time</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:Y1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -6633,7 +6821,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet61.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6664,7 +6852,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet62.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6850,7 +7038,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6891,7 +7079,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet64.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6938,7 +7126,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet65.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6999,7 +7187,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet66.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7050,7 +7238,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7111,7 +7299,133 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>site_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>site_name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>residues</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ligand_interactions</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>conservation_score</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>functional_importance</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>go_terms</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>ec_number</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>protein_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>pdb_entry</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>chain_id</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>residue_range</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>confidence_score</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>evidence_type</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>evidence_code</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>source_database</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>annotation_method</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>publication_ids</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="N2:N1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"experimental,predicted,inferred,literature,author_statement,curator_inference"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7177,7 +7491,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7208,133 +7522,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:U1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>site_type</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>site_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>residues</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>ligand_interactions</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>conservation_score</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>functional_importance</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>go_terms</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>ec_number</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>protein_id</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>pdb_entry</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>chain_id</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>residue_range</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>confidence_score</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>evidence_type</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>evidence_code</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>source_database</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>annotation_method</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>publication_ids</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="N2:N1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"experimental,predicted,inferred,literature,author_statement,curator_inference"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7375,7 +7563,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7401,7 +7589,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7427,7 +7615,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet73.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7468,7 +7656,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet74.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7532,14 +7720,14 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"target,subunit,binding_partner,fusion_partner,chaperone,contaminant,standard"</formula1>
+      <formula1>"target,subunit,binding_partner,fusion_partner,chaperone,carrier,contaminant,standard"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7621,7 +7809,94 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sample_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>subject_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>object_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>interaction_type</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>interaction_status</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>stoichiometry</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>subject_site</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>object_site</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>affinity</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>affinity_type</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"designed,expected,observed,not_observed"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"kd,ki,ic50,ec50,ka,km"</formula1>
+    </dataValidation>
+    <dataValidation sqref="K2:K1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"experimental,predicted,homology,coexpression,colocalization,genetic,physical,functional"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7657,7 +7932,147 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>feature_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>secondary_structure</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>solvent_accessibility</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>backbone_flexibility</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>disorder_probability</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>conformational_state</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>structural_motif</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>domain_assignment</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>domain_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>protein_id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>pdb_entry</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>chain_id</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>residue_range</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>confidence_score</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>evidence_type</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>evidence_code</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>source_database</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>annotation_method</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>publication_ids</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="4">
+    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"alpha_helix,beta_sheet,beta_strand,turn,coil,disordered_region,transmembrane_helix,signal_peptide,transit_peptide,domain,repeat,zinc_finger,zinc_binding,coiled_coil,motif,cavity,channel,pore,hinge,linker"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"helix,sheet,turn,coil,helix_310,helix_pi,bend,bridge"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"open,closed,intermediate,active,inactive,apo,holo,substrate_bound,product_bound,inhibitor_bound,partially_open,partially_closed,disordered"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O2:O1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"experimental,predicted,inferred,literature,author_statement,curator_inference"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet80.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7683,7 +8098,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet81.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7719,7 +8134,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet82.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7755,147 +8170,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:V1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>feature_type</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>secondary_structure</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>solvent_accessibility</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>backbone_flexibility</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>disorder_probability</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>conformational_state</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>structural_motif</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>domain_assignment</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>domain_id</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>protein_id</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>pdb_entry</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>chain_id</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>residue_range</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>confidence_score</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>evidence_type</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>evidence_code</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>source_database</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>annotation_method</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>publication_ids</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="4">
-    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"alpha_helix,beta_sheet,beta_strand,turn,coil,disordered_region,transmembrane_helix,signal_peptide,transit_peptide,domain,repeat,zinc_finger,zinc_binding,coiled_coil,motif,cavity,channel,pore,hinge,linker"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"helix,sheet,turn,coil,helix_310,helix_pi,bend,bridge"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"open,closed,intermediate,active,inactive,apo,holo,substrate_bound,product_bound,inhibitor_bound,partially_open,partially_closed,disordered"</formula1>
-    </dataValidation>
-    <dataValidation sqref="O2:O1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"experimental,predicted,inferred,literature,author_statement,curator_inference"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet80.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet83.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7941,7 +8216,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet81.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet84.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7977,7 +8252,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet82.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet85.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8013,7 +8288,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet83.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet86.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8054,7 +8329,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet84.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet87.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Regenerate artifacts for solution_nmr, nmr_star and the bmrb prefix
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012joHW2nUSe6bVKop3HNaqP
</commit_message>
<xml_diff>
--- a/assets/excel/lambda_ber_schema.xlsx
+++ b/assets/excel/lambda_ber_schema.xlsx
@@ -3738,7 +3738,7 @@
   </sheetData>
   <dataValidations count="4">
     <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"cryo_em,xray_crystallography,saxs,waxs,sans,cryo_et,electron_microscopy,mass_spectrometry,xas,xanes,exafs,xmcd,neutron_crystallography,fiber_diffraction,time_resolved_crystallography,xray_tomography,microed"</formula1>
+      <formula1>"cryo_em,xray_crystallography,saxs,waxs,sans,cryo_et,electron_microscopy,mass_spectrometry,xas,xanes,exafs,xmcd,neutron_crystallography,fiber_diffraction,time_resolved_crystallography,xray_tomography,microed,solution_nmr"</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"SYNCHROTRON_BEAMLINE,NEUTRON_BEAMLINE,XFEL_BEAMLINE,ELECTRON_MICROSCOPE,BENCHTOP_XRAY,OPTICAL_MICROSCOPE,SPECTROMETER"</formula1>
@@ -4025,7 +4025,7 @@
   </sheetData>
   <dataValidations count="8">
     <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"cryo_em,xray_crystallography,saxs,waxs,sans,cryo_et,electron_microscopy,mass_spectrometry,xas,xanes,exafs,xmcd,neutron_crystallography,fiber_diffraction,time_resolved_crystallography,xray_tomography,microed"</formula1>
+      <formula1>"cryo_em,xray_crystallography,saxs,waxs,sans,cryo_et,electron_microscopy,mass_spectrometry,xas,xanes,exafs,xmcd,neutron_crystallography,fiber_diffraction,time_resolved_crystallography,xray_tomography,microed,solution_nmr"</formula1>
     </dataValidation>
     <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"synchrotron,rotating_anode,microfocus,metal_jet"</formula1>
@@ -4478,7 +4478,7 @@
   </sheetData>
   <dataValidations count="5">
     <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"cryo_em,xray_crystallography,saxs,waxs,sans,cryo_et,electron_microscopy,mass_spectrometry,xas,xanes,exafs,xmcd,neutron_crystallography,fiber_diffraction,time_resolved_crystallography,xray_tomography,microed"</formula1>
+      <formula1>"cryo_em,xray_crystallography,saxs,waxs,sans,cryo_et,electron_microscopy,mass_spectrometry,xas,xanes,exafs,xmcd,neutron_crystallography,fiber_diffraction,time_resolved_crystallography,xray_tomography,microed,solution_nmr"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"x_ray_diffraction,neutron_diffraction,electron_diffraction,fiber_diffraction"</formula1>
@@ -4937,7 +4937,7 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"mrc,tiff,hdf5,star,pdb,mmcif,mtz,cbf,cbf_zst,img,h5,ascii,thermo_raw,zip,tar,mrcs,eer,cs,json,csv,ccp4,gz"</formula1>
+      <formula1>"mrc,tiff,hdf5,star,pdb,mmcif,mtz,cbf,cbf_zst,img,h5,ascii,thermo_raw,zip,tar,mrcs,eer,cs,json,csv,ccp4,gz,nmr_star"</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"micrograph,diffraction,scattering,particles,volume,model,metadata,raw_data,processed_data,movie,motion_corrected,ctf_estimation,particle_coordinates,class_averages,fsc_curve,map_half,validation_report"</formula1>

</xml_diff>

<commit_message>
Model particle-to-model inference, structure priors and per-state outputs
Methods such as Fold'EM (arXiv:2610.01358) infer an atomic model straight
from particle images with a structure prediction as prior, skipping the
map. The schema had no way to say so: add workflow types
particle_to_model_inference, structure_prediction and
heterogeneity_analysis; input types particles and structure_prior; data
and output types for predicted models and per-particle assignments;
WorkflowRun.number_of_particles; and conformational_state plus a
per-state particle count on WorkflowOutputAssociation.

Two worked datasets from the paper (integrin a5b1-BIIG2 Fab, UvrA-DNA
two states) and a WorkflowRun example exercise the new terms.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vs1uZSBidJju6qTmq4GkhH
</commit_message>
<xml_diff>
--- a/assets/excel/lambda_ber_schema.xlsx
+++ b/assets/excel/lambda_ber_schema.xlsx
@@ -4503,7 +4503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BP1"/>
+  <dimension ref="A1:BQ1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4829,20 +4829,25 @@
       </c>
       <c r="BM1" t="inlineStr">
         <is>
+          <t>number_of_particles</t>
+        </is>
+      </c>
+      <c r="BN1" t="inlineStr">
+        <is>
           <t>output_files</t>
         </is>
       </c>
-      <c r="BN1" t="inlineStr">
+      <c r="BO1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="BO1" t="inlineStr">
+      <c r="BP1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="BP1" t="inlineStr">
+      <c r="BQ1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -4940,7 +4945,7 @@
       <formula1>"mrc,tiff,hdf5,star,pdb,mmcif,mtz,cbf,cbf_zst,img,h5,ascii,thermo_raw,zip,tar,mrcs,eer,cs,json,csv,ccp4,gz"</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"micrograph,diffraction,scattering,particles,volume,model,metadata,raw_data,processed_data,movie,motion_corrected,ctf_estimation,particle_coordinates,class_averages,fsc_curve,map_half,validation_report"</formula1>
+      <formula1>"micrograph,diffraction,scattering,particles,volume,model,metadata,raw_data,processed_data,movie,motion_corrected,ctf_estimation,particle_coordinates,class_averages,fsc_curve,map_half,validation_report,predicted_model,particle_assignments"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8127,7 +8132,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"raw_data,reference,parameters,mask"</formula1>
+      <formula1>"raw_data,reference,parameters,mask,particles,structure_prior"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8140,7 +8145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8157,13 +8162,23 @@
       <c r="C1" t="inlineStr">
         <is>
           <t>output_type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>conformational_state</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>number_of_particles</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"map,model,particles,micrographs,ctf_estimates,metadata,statistics,processed_data,log"</formula1>
+      <formula1>"map,model,particles,micrographs,ctf_estimates,metadata,statistics,processed_data,log,particle_assignments"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Regenerate artifacts for the cryo-EM terms and profile 0.3.4
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/excel/lambda_ber_schema.xlsx
+++ b/assets/excel/lambda_ber_schema.xlsx
@@ -4095,7 +4095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BW1"/>
+  <dimension ref="A1:CE1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4156,320 +4156,360 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>accelerating_voltage</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>cs</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>magnification</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>nominal_pixel_size</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
         <is>
           <t>calibrated_pixel_size</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>camera_binning</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>exposure_time_per_frame</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>frames_per_movie</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>total_exposure_time</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>total_dose</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>dose_rate</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>spot_size</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>c2_aperture</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>beam_diameter</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>energy_filter_slit_width</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>phase_plate_used</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
         <is>
           <t>defocus_target</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>defocus_range_min</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>defocus_range_max</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>defocus_range_increment</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>astigmatism_target</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>coma</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>stage_tilt</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>tilting_scheme</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>tilt_angle_min</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>tilt_angle_max</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>tilt_angle_increment</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>tilt_axis_angle</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>number_of_tilt_images</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>dose_per_tilt</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>dual_tilt_axis_rotation</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>fiducial_size</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>rotation_rate</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>camera_length</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>frames_per_second</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>autoloader_slot</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>shots_per_hole</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>holes_per_group</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>acquisition_software</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>acquisition_software_version</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>detector</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>wavelength</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>energy</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>oscillation_angle</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>start_angle</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>sweep_start</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>sweep_end</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>number_of_images</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>beam_center_x</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>beam_center_y</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>beam_center_pixels</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>detector_distance</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>pixel_size_x</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>pixel_size_y</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
         <is>
           <t>total_rotation</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BO1" t="inlineStr">
         <is>
           <t>transmission</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BP1" t="inlineStr">
         <is>
           <t>flux</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BQ1" t="inlineStr">
         <is>
           <t>flux_end</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BR1" t="inlineStr">
         <is>
           <t>slit_gap_horizontal</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BS1" t="inlineStr">
         <is>
           <t>slit_gap_vertical</t>
         </is>
       </c>
-      <c r="BL1" t="inlineStr">
+      <c r="BT1" t="inlineStr">
         <is>
           <t>undulator_gap</t>
         </is>
       </c>
-      <c r="BM1" t="inlineStr">
+      <c r="BU1" t="inlineStr">
         <is>
           <t>synchrotron_mode</t>
         </is>
       </c>
-      <c r="BN1" t="inlineStr">
+      <c r="BV1" t="inlineStr">
         <is>
           <t>exposure_time</t>
         </is>
       </c>
-      <c r="BO1" t="inlineStr">
+      <c r="BW1" t="inlineStr">
         <is>
           <t>start_time</t>
         </is>
       </c>
-      <c r="BP1" t="inlineStr">
+      <c r="BX1" t="inlineStr">
         <is>
           <t>end_time</t>
         </is>
       </c>
-      <c r="BQ1" t="inlineStr">
+      <c r="BY1" t="inlineStr">
         <is>
           <t>resolution</t>
         </is>
       </c>
-      <c r="BR1" t="inlineStr">
+      <c r="BZ1" t="inlineStr">
         <is>
           <t>resolution_at_corner</t>
         </is>
       </c>
-      <c r="BS1" t="inlineStr">
+      <c r="CA1" t="inlineStr">
         <is>
           <t>ispyb_data_collection_id</t>
         </is>
       </c>
-      <c r="BT1" t="inlineStr">
+      <c r="CB1" t="inlineStr">
         <is>
           <t>ispyb_session_id</t>
         </is>
       </c>
-      <c r="BU1" t="inlineStr">
+      <c r="CC1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="BV1" t="inlineStr">
+      <c r="CD1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="BW1" t="inlineStr">
+      <c r="CE1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -4489,7 +4529,7 @@
     <dataValidation sqref="K2:K1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"bluesky,spec,sardana,gda,mxcube_daq,blu_ice,jblue_ice"</formula1>
     </dataValidation>
-    <dataValidation sqref="AA2:AA1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AI2:AI1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"none,dose_symmetric,linear,continuous"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4937,10 +4977,10 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"mrc,tiff,hdf5,star,pdb,mmcif,mtz,cbf,cbf_zst,img,h5,ascii,thermo_raw,zip,tar,mrcs,eer,cs,json,csv,ccp4,gz"</formula1>
+      <formula1>"mrc,tiff,hdf5,star,pdb,mmcif,mtz,cbf,cbf_zst,img,h5,ascii,thermo_raw,zip,tar,mrcs,eer,cs,json,csv,ccp4,gz,yaml,mdoc,nav,dm4"</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"micrograph,diffraction,scattering,particles,volume,model,metadata,raw_data,processed_data,movie,motion_corrected,ctf_estimation,particle_coordinates,class_averages,fsc_curve,map_half,validation_report"</formula1>
+      <formula1>"micrograph,diffraction,scattering,particles,volume,model,metadata,raw_data,processed_data,movie,motion_corrected,ctf_estimation,particle_coordinates,class_averages,fsc_curve,map_half,validation_report,gain_reference,defect_map,atlas,screening_image"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Regenerate artifacts for instrument_type
Refs #128

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/excel/lambda_ber_schema.xlsx
+++ b/assets/excel/lambda_ber_schema.xlsx
@@ -2921,76 +2921,81 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>instrument_type</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>instrument_code</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>instrument_registry_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>instrument_category</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>facility_name</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>facility_ror</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>facility_organization_id</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>beamline_id</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>installation_date</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -2998,13 +3003,13 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"SYNCHROTRON_BEAMLINE,NEUTRON_BEAMLINE,XFEL_BEAMLINE,ELECTRON_MICROSCOPE,BENCHTOP_XRAY,OPTICAL_MICROSCOPE,SPECTROMETER"</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"operational,maintenance,offline,commissioning"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3018,7 +3023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN1"/>
+  <dimension ref="A1:AO1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3154,70 +3159,75 @@
       </c>
       <c r="AA1" t="inlineStr">
         <is>
+          <t>instrument_type</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
           <t>instrument_code</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>instrument_registry_id</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>instrument_category</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>facility_name</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>facility_ror</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>facility_organization_id</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>beamline_id</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>installation_date</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3234,13 +3244,13 @@
     <dataValidation sqref="Y2:Y1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"EFTEM,TEM,STEM"</formula1>
     </dataValidation>
-    <dataValidation sqref="AC2:AC1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AD2:AD1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"SYNCHROTRON_BEAMLINE,NEUTRON_BEAMLINE,XFEL_BEAMLINE,ELECTRON_MICROSCOPE,BENCHTOP_XRAY,OPTICAL_MICROSCOPE,SPECTROMETER"</formula1>
     </dataValidation>
-    <dataValidation sqref="AD2:AD1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AE2:AE1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
     </dataValidation>
-    <dataValidation sqref="AK2:AK1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="AL2:AL1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"operational,maintenance,offline,commissioning"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3254,7 +3264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1"/>
+  <dimension ref="A1:AA1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3320,70 +3330,75 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>instrument_type</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>instrument_code</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>instrument_registry_id</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>instrument_category</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>facility_name</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>facility_ror</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>facility_organization_id</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>beamline_id</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>installation_date</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3397,13 +3412,13 @@
     <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"direct_electron_detector,ccd,cmos,hybrid_photon_counting,scintillator_coupled,imaging_plate,film"</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="P2:P1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"SYNCHROTRON_BEAMLINE,NEUTRON_BEAMLINE,XFEL_BEAMLINE,ELECTRON_MICROSCOPE,BENCHTOP_XRAY,OPTICAL_MICROSCOPE,SPECTROMETER"</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Q2:Q1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
     </dataValidation>
-    <dataValidation sqref="W2:W1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="X2:X1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"operational,maintenance,offline,commissioning"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3625,7 +3640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U1"/>
+  <dimension ref="A1:V1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3666,70 +3681,75 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>instrument_type</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>instrument_code</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>instrument_registry_id</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>instrument_category</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>facility_name</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>facility_ror</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>facility_organization_id</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>beamline_id</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>installation_date</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3740,13 +3760,13 @@
     <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"cryo_em,xray_crystallography,saxs,waxs,sans,cryo_et,electron_microscopy,mass_spectrometry,xas,xanes,exafs,xmcd,neutron_crystallography,fiber_diffraction,time_resolved_crystallography,xray_tomography,microed"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"SYNCHROTRON_BEAMLINE,NEUTRON_BEAMLINE,XFEL_BEAMLINE,ELECTRON_MICROSCOPE,BENCHTOP_XRAY,OPTICAL_MICROSCOPE,SPECTROMETER"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
     </dataValidation>
-    <dataValidation sqref="R2:R1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="S2:S1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"operational,maintenance,offline,commissioning"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3760,7 +3780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1"/>
+  <dimension ref="A1:U1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3796,70 +3816,75 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>instrument_type</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>instrument_code</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>instrument_registry_id</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>instrument_category</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>facility_name</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>facility_ror</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>facility_organization_id</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>beamline_id</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>installation_date</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3867,13 +3892,13 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="I2:I1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"SYNCHROTRON_BEAMLINE,NEUTRON_BEAMLINE,XFEL_BEAMLINE,ELECTRON_MICROSCOPE,BENCHTOP_XRAY,OPTICAL_MICROSCOPE,SPECTROMETER"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K2:K1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q2:Q1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="R2:R1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"operational,maintenance,offline,commissioning"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3887,7 +3912,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1"/>
+  <dimension ref="A1:AA1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3953,70 +3978,75 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>instrument_type</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>instrument_code</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>instrument_registry_id</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>instrument_category</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>facility_name</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>facility_ror</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>facility_organization_id</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>beamline_id</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>model</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>installation_date</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>current_status</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -4039,13 +4069,13 @@
     <dataValidation sqref="L2:L1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"epics,tango,labview,opi"</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="P2:P1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"SYNCHROTRON_BEAMLINE,NEUTRON_BEAMLINE,XFEL_BEAMLINE,ELECTRON_MICROSCOPE,BENCHTOP_XRAY,OPTICAL_MICROSCOPE,SPECTROMETER"</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Q2:Q1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"NSLS_II,ALS,SSRL,ESRF,DIAMOND,PHOTON_FACTORY,APS,SPRING8,PETRA_III,SOLEIL,AUSTRALIAN_SYNCHROTRON,EMSL,SNS,HFIR"</formula1>
     </dataValidation>
-    <dataValidation sqref="W2:W1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="X2:X1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"operational,maintenance,offline,commissioning"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>